<commit_message>
Add tracked model promotion and daily Docker pipeline
</commit_message>
<xml_diff>
--- a/data/processed/predicciones.xlsx
+++ b/data/processed/predicciones.xlsx
@@ -523,40 +523,40 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B2" t="n">
+        <v>33</v>
+      </c>
+      <c r="C2" t="n">
         <v>43</v>
       </c>
-      <c r="C2" t="n">
-        <v>34</v>
-      </c>
       <c r="D2" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="E2" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F2" t="n">
         <v>34</v>
       </c>
       <c r="G2" t="n">
+        <v>34</v>
+      </c>
+      <c r="H2" t="n">
         <v>29</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>48</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>40</v>
       </c>
-      <c r="J2" t="n">
-        <v>46</v>
-      </c>
       <c r="K2" t="n">
+        <v>46</v>
+      </c>
+      <c r="L2" t="n">
         <v>41</v>
-      </c>
-      <c r="L2" t="n">
-        <v>49</v>
       </c>
       <c r="M2" t="n">
         <v>36.66666666666666</v>
@@ -565,16 +565,16 @@
         <v>38</v>
       </c>
       <c r="O2" t="n">
-        <v>36.55554040022041</v>
+        <v>35.2777702001102</v>
       </c>
       <c r="P2" t="n">
-        <v>37.5025287839951</v>
+        <v>36.33501918933007</v>
       </c>
       <c r="Q2" t="n">
         <v>34</v>
       </c>
       <c r="R2" t="n">
-        <v>47.21984385134578</v>
+        <v>42.58569749513992</v>
       </c>
     </row>
     <row r="3">
@@ -582,391 +582,391 @@
         <v>34</v>
       </c>
       <c r="B3" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C3" t="n">
+        <v>33</v>
+      </c>
+      <c r="D3" t="n">
         <v>43</v>
       </c>
-      <c r="D3" t="n">
-        <v>34</v>
-      </c>
       <c r="E3" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="F3" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="G3" t="n">
         <v>34</v>
       </c>
       <c r="H3" t="n">
+        <v>34</v>
+      </c>
+      <c r="I3" t="n">
         <v>29</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>48</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>40</v>
       </c>
-      <c r="K3" t="n">
-        <v>46</v>
-      </c>
       <c r="L3" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="M3" t="n">
-        <v>36.66666666666666</v>
+        <v>33.66666666666666</v>
       </c>
       <c r="N3" t="n">
-        <v>38</v>
+        <v>35.6</v>
       </c>
       <c r="O3" t="n">
-        <v>35.2777702001102</v>
+        <v>34.63888510005511</v>
       </c>
       <c r="P3" t="n">
-        <v>36.33501918933007</v>
+        <v>35.55667945955338</v>
       </c>
       <c r="Q3" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="R3" t="n">
-        <v>42.63015643484845</v>
+        <v>42.49577911475136</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B4" t="n">
         <v>34</v>
       </c>
       <c r="C4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D4" t="n">
+        <v>33</v>
+      </c>
+      <c r="E4" t="n">
         <v>43</v>
       </c>
-      <c r="E4" t="n">
-        <v>34</v>
-      </c>
       <c r="F4" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="G4" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H4" t="n">
         <v>34</v>
       </c>
       <c r="I4" t="n">
+        <v>34</v>
+      </c>
+      <c r="J4" t="n">
         <v>29</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>48</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>40</v>
       </c>
-      <c r="L4" t="n">
-        <v>46</v>
-      </c>
       <c r="M4" t="n">
-        <v>33.66666666666666</v>
+        <v>38</v>
       </c>
       <c r="N4" t="n">
-        <v>35.6</v>
+        <v>38</v>
       </c>
       <c r="O4" t="n">
-        <v>34.63888510005511</v>
+        <v>40.31944255002755</v>
       </c>
       <c r="P4" t="n">
-        <v>35.55667945955338</v>
+        <v>39.03778630636892</v>
       </c>
       <c r="Q4" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="R4" t="n">
-        <v>42.53926441079397</v>
+        <v>44.76076020626862</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B5" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C5" t="n">
         <v>34</v>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E5" t="n">
+        <v>33</v>
+      </c>
+      <c r="F5" t="n">
         <v>43</v>
       </c>
-      <c r="F5" t="n">
-        <v>34</v>
-      </c>
       <c r="G5" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="H5" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="I5" t="n">
         <v>34</v>
       </c>
       <c r="J5" t="n">
+        <v>34</v>
+      </c>
+      <c r="K5" t="n">
         <v>29</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>48</v>
       </c>
-      <c r="L5" t="n">
-        <v>40</v>
-      </c>
       <c r="M5" t="n">
+        <v>36.33333333333334</v>
+      </c>
+      <c r="N5" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="O5" t="n">
+        <v>34.65972127501378</v>
+      </c>
+      <c r="P5" t="n">
+        <v>35.69185753757928</v>
+      </c>
+      <c r="Q5" t="n">
         <v>38</v>
       </c>
-      <c r="N5" t="n">
-        <v>38</v>
-      </c>
-      <c r="O5" t="n">
-        <v>40.31944255002755</v>
-      </c>
-      <c r="P5" t="n">
-        <v>39.03778630636892</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>29</v>
-      </c>
       <c r="R5" t="n">
-        <v>44.78793153854507</v>
+        <v>38.81327062676211</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B6" t="n">
         <v>29</v>
       </c>
-      <c r="B6" t="n">
-        <v>46</v>
-      </c>
       <c r="C6" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="D6" t="n">
         <v>34</v>
       </c>
       <c r="E6" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F6" t="n">
+        <v>33</v>
+      </c>
+      <c r="G6" t="n">
         <v>43</v>
       </c>
-      <c r="G6" t="n">
-        <v>34</v>
-      </c>
       <c r="H6" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="I6" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="J6" t="n">
         <v>34</v>
       </c>
       <c r="K6" t="n">
+        <v>34</v>
+      </c>
+      <c r="L6" t="n">
         <v>29</v>
       </c>
-      <c r="L6" t="n">
-        <v>48</v>
-      </c>
       <c r="M6" t="n">
-        <v>36.33333333333334</v>
+        <v>37.66666666666666</v>
       </c>
       <c r="N6" t="n">
-        <v>35.2</v>
+        <v>36.2</v>
       </c>
       <c r="O6" t="n">
-        <v>34.65972127501378</v>
+        <v>36.32986063750689</v>
       </c>
       <c r="P6" t="n">
-        <v>35.69185753757928</v>
+        <v>36.46123835838619</v>
       </c>
       <c r="Q6" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="R6" t="n">
-        <v>38.8571716370659</v>
+        <v>43.08960212996828</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
+        <v>36</v>
+      </c>
+      <c r="B7" t="n">
         <v>38</v>
       </c>
-      <c r="B7" t="n">
+      <c r="C7" t="n">
         <v>29</v>
       </c>
-      <c r="C7" t="n">
-        <v>46</v>
-      </c>
       <c r="D7" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="E7" t="n">
         <v>34</v>
       </c>
       <c r="F7" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G7" t="n">
+        <v>33</v>
+      </c>
+      <c r="H7" t="n">
         <v>43</v>
       </c>
-      <c r="H7" t="n">
-        <v>34</v>
-      </c>
       <c r="I7" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="J7" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K7" t="n">
         <v>34</v>
       </c>
       <c r="L7" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="M7" t="n">
-        <v>37.66666666666666</v>
+        <v>34.33333333333334</v>
       </c>
       <c r="N7" t="n">
-        <v>36.2</v>
+        <v>36.6</v>
       </c>
       <c r="O7" t="n">
-        <v>36.32986063750689</v>
+        <v>36.16493031875345</v>
       </c>
       <c r="P7" t="n">
-        <v>36.46123835838619</v>
+        <v>36.30749223892413</v>
       </c>
       <c r="Q7" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="R7" t="n">
-        <v>43.12375153921106</v>
+        <v>43.44869782376701</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>33</v>
+      </c>
+      <c r="B8" t="n">
         <v>36</v>
       </c>
-      <c r="B8" t="n">
+      <c r="C8" t="n">
         <v>38</v>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="n">
         <v>29</v>
       </c>
-      <c r="D8" t="n">
-        <v>46</v>
-      </c>
       <c r="E8" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="F8" t="n">
         <v>34</v>
       </c>
       <c r="G8" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H8" t="n">
+        <v>33</v>
+      </c>
+      <c r="I8" t="n">
         <v>43</v>
       </c>
-      <c r="I8" t="n">
-        <v>34</v>
-      </c>
       <c r="J8" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="K8" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="L8" t="n">
         <v>34</v>
       </c>
       <c r="M8" t="n">
-        <v>34.33333333333334</v>
+        <v>35.66666666666666</v>
       </c>
       <c r="N8" t="n">
-        <v>36.6</v>
+        <v>36.4</v>
       </c>
       <c r="O8" t="n">
-        <v>36.16493031875345</v>
+        <v>34.58246515937672</v>
       </c>
       <c r="P8" t="n">
-        <v>36.30749223892413</v>
+        <v>35.20499482594942</v>
       </c>
       <c r="Q8" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R8" t="n">
-        <v>43.4924042322325</v>
+        <v>39.06033662598349</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" t="n">
+        <v>33</v>
+      </c>
+      <c r="C9" t="n">
         <v>36</v>
       </c>
-      <c r="C9" t="n">
+      <c r="D9" t="n">
         <v>38</v>
       </c>
-      <c r="D9" t="n">
+      <c r="E9" t="n">
         <v>29</v>
       </c>
-      <c r="E9" t="n">
-        <v>46</v>
-      </c>
       <c r="F9" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="G9" t="n">
         <v>34</v>
       </c>
       <c r="H9" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I9" t="n">
+        <v>33</v>
+      </c>
+      <c r="J9" t="n">
         <v>43</v>
       </c>
-      <c r="J9" t="n">
-        <v>34</v>
-      </c>
       <c r="K9" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="L9" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="M9" t="n">
-        <v>35.66666666666666</v>
+        <v>33.66666666666666</v>
       </c>
       <c r="N9" t="n">
-        <v>36.4</v>
+        <v>33.6</v>
       </c>
       <c r="O9" t="n">
-        <v>34.58246515937672</v>
+        <v>33.29123257968836</v>
       </c>
       <c r="P9" t="n">
-        <v>35.20499482594942</v>
+        <v>34.13666321729961</v>
       </c>
       <c r="Q9" t="n">
         <v>32</v>
       </c>
       <c r="R9" t="n">
-        <v>39.08711303722315</v>
+        <v>40.78555089418443</v>
       </c>
     </row>
     <row r="10">
@@ -974,391 +974,391 @@
         <v>32</v>
       </c>
       <c r="B10" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C10" t="n">
+        <v>33</v>
+      </c>
+      <c r="D10" t="n">
         <v>36</v>
       </c>
-      <c r="D10" t="n">
+      <c r="E10" t="n">
         <v>38</v>
       </c>
-      <c r="E10" t="n">
+      <c r="F10" t="n">
         <v>29</v>
       </c>
-      <c r="F10" t="n">
-        <v>46</v>
-      </c>
       <c r="G10" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="H10" t="n">
         <v>34</v>
       </c>
       <c r="I10" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="J10" t="n">
+        <v>33</v>
+      </c>
+      <c r="K10" t="n">
         <v>43</v>
       </c>
-      <c r="K10" t="n">
-        <v>34</v>
-      </c>
       <c r="L10" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="M10" t="n">
-        <v>33.66666666666666</v>
+        <v>32.33333333333334</v>
       </c>
       <c r="N10" t="n">
-        <v>33.6</v>
+        <v>34.2</v>
       </c>
       <c r="O10" t="n">
-        <v>33.29123257968836</v>
+        <v>32.64561628984418</v>
       </c>
       <c r="P10" t="n">
-        <v>34.13666321729961</v>
+        <v>33.42444214486641</v>
       </c>
       <c r="Q10" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="R10" t="n">
-        <v>40.82194599215813</v>
+        <v>39.62207056268527</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B11" t="n">
         <v>32</v>
       </c>
       <c r="C11" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D11" t="n">
+        <v>33</v>
+      </c>
+      <c r="E11" t="n">
         <v>36</v>
       </c>
-      <c r="E11" t="n">
+      <c r="F11" t="n">
         <v>38</v>
       </c>
-      <c r="F11" t="n">
+      <c r="G11" t="n">
         <v>29</v>
       </c>
-      <c r="G11" t="n">
-        <v>46</v>
-      </c>
       <c r="H11" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="I11" t="n">
         <v>34</v>
       </c>
       <c r="J11" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K11" t="n">
+        <v>33</v>
+      </c>
+      <c r="L11" t="n">
         <v>43</v>
       </c>
-      <c r="L11" t="n">
-        <v>34</v>
-      </c>
       <c r="M11" t="n">
-        <v>32.33333333333334</v>
+        <v>33</v>
       </c>
       <c r="N11" t="n">
-        <v>34.2</v>
+        <v>33.6</v>
       </c>
       <c r="O11" t="n">
-        <v>32.64561628984418</v>
+        <v>33.82280814492209</v>
       </c>
       <c r="P11" t="n">
-        <v>33.42444214486641</v>
+        <v>33.94962809657761</v>
       </c>
       <c r="Q11" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="R11" t="n">
-        <v>39.665895712287</v>
+        <v>42.15045351175433</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B12" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C12" t="n">
         <v>32</v>
       </c>
       <c r="D12" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" t="n">
+        <v>33</v>
+      </c>
+      <c r="F12" t="n">
         <v>36</v>
       </c>
-      <c r="F12" t="n">
+      <c r="G12" t="n">
         <v>38</v>
       </c>
-      <c r="G12" t="n">
+      <c r="H12" t="n">
         <v>29</v>
       </c>
-      <c r="H12" t="n">
-        <v>46</v>
-      </c>
       <c r="I12" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="J12" t="n">
         <v>34</v>
       </c>
       <c r="K12" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="L12" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="M12" t="n">
-        <v>30.66666666666667</v>
+        <v>34.66666666666666</v>
       </c>
       <c r="N12" t="n">
-        <v>32.2</v>
+        <v>33.8</v>
       </c>
       <c r="O12" t="n">
-        <v>30.32280814492209</v>
+        <v>35.41140407246105</v>
       </c>
       <c r="P12" t="n">
-        <v>31.61629476324428</v>
+        <v>34.96641873105175</v>
       </c>
       <c r="Q12" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="R12" t="n">
-        <v>38.6819026830833</v>
+        <v>43.01709913970409</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
+        <v>36</v>
+      </c>
+      <c r="B13" t="n">
         <v>37</v>
       </c>
-      <c r="B13" t="n">
-        <v>28</v>
-      </c>
       <c r="C13" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D13" t="n">
         <v>32</v>
       </c>
       <c r="E13" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F13" t="n">
+        <v>33</v>
+      </c>
+      <c r="G13" t="n">
         <v>36</v>
       </c>
-      <c r="G13" t="n">
+      <c r="H13" t="n">
         <v>38</v>
       </c>
-      <c r="H13" t="n">
+      <c r="I13" t="n">
         <v>29</v>
       </c>
-      <c r="I13" t="n">
-        <v>46</v>
-      </c>
       <c r="J13" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="K13" t="n">
         <v>34</v>
       </c>
       <c r="L13" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M13" t="n">
-        <v>32.33333333333334</v>
+        <v>36</v>
       </c>
       <c r="N13" t="n">
-        <v>32.4</v>
+        <v>34.4</v>
       </c>
       <c r="O13" t="n">
-        <v>33.66140407246105</v>
+        <v>35.70570203623052</v>
       </c>
       <c r="P13" t="n">
-        <v>33.41086317549619</v>
+        <v>35.31094582070116</v>
       </c>
       <c r="Q13" t="n">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="R13" t="n">
-        <v>42.91051714433865</v>
+        <v>43.90066152073415</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
+        <v>48</v>
+      </c>
+      <c r="B14" t="n">
+        <v>36</v>
+      </c>
+      <c r="C14" t="n">
+        <v>37</v>
+      </c>
+      <c r="D14" t="n">
         <v>35</v>
-      </c>
-      <c r="B14" t="n">
-        <v>37</v>
-      </c>
-      <c r="C14" t="n">
-        <v>28</v>
-      </c>
-      <c r="D14" t="n">
-        <v>32</v>
       </c>
       <c r="E14" t="n">
         <v>32</v>
       </c>
       <c r="F14" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G14" t="n">
+        <v>33</v>
+      </c>
+      <c r="H14" t="n">
         <v>36</v>
       </c>
-      <c r="H14" t="n">
+      <c r="I14" t="n">
         <v>38</v>
       </c>
-      <c r="I14" t="n">
+      <c r="J14" t="n">
         <v>29</v>
       </c>
-      <c r="J14" t="n">
-        <v>46</v>
-      </c>
       <c r="K14" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="L14" t="n">
         <v>34</v>
       </c>
       <c r="M14" t="n">
-        <v>33.33333333333334</v>
+        <v>40.33333333333334</v>
       </c>
       <c r="N14" t="n">
-        <v>32.8</v>
+        <v>37.6</v>
       </c>
       <c r="O14" t="n">
-        <v>34.33070203623052</v>
+        <v>41.85285101811526</v>
       </c>
       <c r="P14" t="n">
-        <v>33.9405754503308</v>
+        <v>39.54063054713411</v>
       </c>
       <c r="Q14" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="R14" t="n">
-        <v>43.37848447278883</v>
+        <v>46.75374272494388</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="B15" t="n">
+        <v>48</v>
+      </c>
+      <c r="C15" t="n">
+        <v>36</v>
+      </c>
+      <c r="D15" t="n">
+        <v>37</v>
+      </c>
+      <c r="E15" t="n">
         <v>35</v>
-      </c>
-      <c r="C15" t="n">
-        <v>37</v>
-      </c>
-      <c r="D15" t="n">
-        <v>28</v>
-      </c>
-      <c r="E15" t="n">
-        <v>32</v>
       </c>
       <c r="F15" t="n">
         <v>32</v>
       </c>
       <c r="G15" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H15" t="n">
+        <v>33</v>
+      </c>
+      <c r="I15" t="n">
         <v>36</v>
       </c>
-      <c r="I15" t="n">
+      <c r="J15" t="n">
         <v>38</v>
       </c>
-      <c r="J15" t="n">
+      <c r="K15" t="n">
         <v>29</v>
       </c>
-      <c r="K15" t="n">
-        <v>46</v>
-      </c>
       <c r="L15" t="n">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="M15" t="n">
-        <v>39.33333333333334</v>
+        <v>37.33333333333334</v>
       </c>
       <c r="N15" t="n">
-        <v>35.6</v>
+        <v>36.8</v>
       </c>
       <c r="O15" t="n">
-        <v>40.16535101811526</v>
+        <v>34.92642550905763</v>
       </c>
       <c r="P15" t="n">
-        <v>37.96038363355387</v>
+        <v>35.69375369808941</v>
       </c>
       <c r="Q15" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="R15" t="n">
-        <v>45.58798777182141</v>
+        <v>39.21400447807752</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
+        <v>30</v>
+      </c>
+      <c r="B16" t="n">
         <v>28</v>
       </c>
-      <c r="B16" t="n">
-        <v>46</v>
-      </c>
       <c r="C16" t="n">
+        <v>48</v>
+      </c>
+      <c r="D16" t="n">
+        <v>36</v>
+      </c>
+      <c r="E16" t="n">
+        <v>37</v>
+      </c>
+      <c r="F16" t="n">
         <v>35</v>
-      </c>
-      <c r="D16" t="n">
-        <v>37</v>
-      </c>
-      <c r="E16" t="n">
-        <v>28</v>
-      </c>
-      <c r="F16" t="n">
-        <v>32</v>
       </c>
       <c r="G16" t="n">
         <v>32</v>
       </c>
       <c r="H16" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I16" t="n">
+        <v>33</v>
+      </c>
+      <c r="J16" t="n">
         <v>36</v>
       </c>
-      <c r="J16" t="n">
+      <c r="K16" t="n">
         <v>38</v>
       </c>
-      <c r="K16" t="n">
+      <c r="L16" t="n">
         <v>29</v>
       </c>
-      <c r="L16" t="n">
-        <v>46</v>
-      </c>
       <c r="M16" t="n">
-        <v>36.33333333333334</v>
+        <v>35.33333333333334</v>
       </c>
       <c r="N16" t="n">
-        <v>34.8</v>
+        <v>35.8</v>
       </c>
       <c r="O16" t="n">
-        <v>34.08267550905763</v>
+        <v>32.46321275452881</v>
       </c>
       <c r="P16" t="n">
-        <v>34.64025575570258</v>
+        <v>33.79583579872627</v>
       </c>
       <c r="Q16" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="R16" t="n">
-        <v>39.14458180802034</v>
+        <v>40.18078324971645</v>
       </c>
     </row>
   </sheetData>
@@ -1409,16 +1409,16 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>60.0112676056338</v>
+        <v>59.97468354430379</v>
       </c>
       <c r="C2" t="n">
-        <v>4.745559381010756e-267</v>
+        <v>2.051178579862612e-267</v>
       </c>
       <c r="D2" t="n">
-        <v>57.96764897234998</v>
+        <v>57.93364403815164</v>
       </c>
       <c r="E2" t="n">
-        <v>62.05488623891761</v>
+        <v>62.01572305045595</v>
       </c>
     </row>
     <row r="3">
@@ -1428,16 +1428,16 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>-21879.83975369471</v>
+        <v>-21684.88753453303</v>
       </c>
       <c r="C3" t="n">
-        <v>0.02392066807263437</v>
+        <v>0.02496443821080301</v>
       </c>
       <c r="D3" t="n">
-        <v>-40859.75046563402</v>
+        <v>-40634.21056466443</v>
       </c>
       <c r="E3" t="n">
-        <v>-2899.929041755404</v>
+        <v>-2735.564504401627</v>
       </c>
     </row>
     <row r="4">
@@ -1447,16 +1447,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>-7206.927025113661</v>
+        <v>-7141.647998520871</v>
       </c>
       <c r="C4" t="n">
-        <v>0.02357781342866415</v>
+        <v>0.02461025114635123</v>
       </c>
       <c r="D4" t="n">
-        <v>-13443.30472141227</v>
+        <v>-13367.00635902572</v>
       </c>
       <c r="E4" t="n">
-        <v>-970.5493288150501</v>
+        <v>-916.2896380160264</v>
       </c>
     </row>
     <row r="5">
@@ -1466,16 +1466,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>102.7520856032184</v>
+        <v>100.577922631512</v>
       </c>
       <c r="C5" t="n">
-        <v>0.05063934407986799</v>
+        <v>0.05278085378303413</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.286807076937464</v>
+        <v>-1.210974287850235</v>
       </c>
       <c r="E5" t="n">
-        <v>205.7909782833744</v>
+        <v>202.3668195508742</v>
       </c>
     </row>
     <row r="6">
@@ -1485,16 +1485,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>-1207.571809788566</v>
+        <v>-1196.931038521037</v>
       </c>
       <c r="C6" t="n">
-        <v>0.02243994405514925</v>
+        <v>0.02344003625953886</v>
       </c>
       <c r="D6" t="n">
-        <v>-2243.838883443532</v>
+        <v>-2231.6432401103</v>
       </c>
       <c r="E6" t="n">
-        <v>-171.3047361335998</v>
+        <v>-162.2188369317741</v>
       </c>
     </row>
     <row r="7">
@@ -1504,16 +1504,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>592.8785772358259</v>
+        <v>586.9633004202778</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0261736905766597</v>
+        <v>0.02728158621028817</v>
       </c>
       <c r="D7" t="n">
-        <v>70.50679081837166</v>
+        <v>66.00371037106152</v>
       </c>
       <c r="E7" t="n">
-        <v>1115.25036365328</v>
+        <v>1107.922890469494</v>
       </c>
     </row>
     <row r="8">
@@ -1523,16 +1523,16 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>-851.4191374920013</v>
+        <v>-843.7199226240964</v>
       </c>
       <c r="C8" t="n">
-        <v>0.02240739794170418</v>
+        <v>0.02340705122613649</v>
       </c>
       <c r="D8" t="n">
-        <v>-1581.879437795159</v>
+        <v>-1572.917178119492</v>
       </c>
       <c r="E8" t="n">
-        <v>-120.958837188844</v>
+        <v>-114.5226671287011</v>
       </c>
     </row>
     <row r="9">
@@ -1542,16 +1542,16 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>-413.6633050197345</v>
+        <v>-409.9820522631182</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02145559261746437</v>
+        <v>0.02242715666904951</v>
       </c>
       <c r="D9" t="n">
-        <v>-766.0059735070563</v>
+        <v>-761.7712013821804</v>
       </c>
       <c r="E9" t="n">
-        <v>-61.32063653241272</v>
+        <v>-58.19290314405612</v>
       </c>
     </row>
     <row r="10">
@@ -1561,16 +1561,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>-196.3175033682553</v>
+        <v>-194.4648159905006</v>
       </c>
       <c r="C10" t="n">
-        <v>0.02178548750787767</v>
+        <v>0.02277153044915444</v>
       </c>
       <c r="D10" t="n">
-        <v>-363.9563858862912</v>
+        <v>-361.7544681003438</v>
       </c>
       <c r="E10" t="n">
-        <v>-28.67862085021937</v>
+        <v>-27.17516388065738</v>
       </c>
     </row>
     <row r="11">
@@ -1580,16 +1580,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-92.57261281964213</v>
+        <v>-91.69827928128578</v>
       </c>
       <c r="C11" t="n">
-        <v>0.02040413025631339</v>
+        <v>0.02136050161329965</v>
       </c>
       <c r="D11" t="n">
-        <v>-170.7751742666767</v>
+        <v>-169.746174164813</v>
       </c>
       <c r="E11" t="n">
-        <v>-14.37005137260753</v>
+        <v>-13.65038439775857</v>
       </c>
     </row>
     <row r="12">
@@ -1599,16 +1599,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-37.64942657091987</v>
+        <v>-37.24866064885972</v>
       </c>
       <c r="C12" t="n">
-        <v>0.03741876386314655</v>
+        <v>0.03907184775191381</v>
       </c>
       <c r="D12" t="n">
-        <v>-73.0999956265982</v>
+        <v>-72.62428348290481</v>
       </c>
       <c r="E12" t="n">
-        <v>-2.198857515241542</v>
+        <v>-1.873037814814616</v>
       </c>
     </row>
     <row r="13">
@@ -1618,16 +1618,16 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>-20.8576164464071</v>
+        <v>-20.67227846400147</v>
       </c>
       <c r="C13" t="n">
-        <v>0.008231919592870859</v>
+        <v>0.008674492780750307</v>
       </c>
       <c r="D13" t="n">
-        <v>-36.31092740530133</v>
+        <v>-36.09259337453565</v>
       </c>
       <c r="E13" t="n">
-        <v>-5.404305487512865</v>
+        <v>-5.2519635534673</v>
       </c>
     </row>
     <row r="14">
@@ -1637,16 +1637,16 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>-8.041751934603649</v>
+        <v>-7.952618459546684</v>
       </c>
       <c r="C14" t="n">
-        <v>0.03480290717699529</v>
+        <v>0.03643326853224146</v>
       </c>
       <c r="D14" t="n">
-        <v>-15.5077481590629</v>
+        <v>-15.40166607888722</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.5757557101444037</v>
+        <v>-0.5035708402061472</v>
       </c>
     </row>
     <row r="15">
@@ -1656,16 +1656,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>-11971.90889045888</v>
+        <v>-11863.7081711499</v>
       </c>
       <c r="C15" t="n">
-        <v>0.02376993675941483</v>
+        <v>0.02480899641612121</v>
       </c>
       <c r="D15" t="n">
-        <v>-22345.88729062254</v>
+        <v>-22219.62210133566</v>
       </c>
       <c r="E15" t="n">
-        <v>-1597.930490295215</v>
+        <v>-1507.794240964153</v>
       </c>
     </row>
     <row r="16">
@@ -1675,16 +1675,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>-8316.651162011744</v>
+        <v>-8240.977140189487</v>
       </c>
       <c r="C16" t="n">
-        <v>0.02366859652078305</v>
+        <v>0.02470477069622849</v>
       </c>
       <c r="D16" t="n">
-        <v>-15518.01154418448</v>
+        <v>-15429.3628905855</v>
       </c>
       <c r="E16" t="n">
-        <v>-1115.290779839006</v>
+        <v>-1052.591389793474</v>
       </c>
     </row>
     <row r="17">
@@ -1694,16 +1694,16 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>46283.36892646742</v>
+        <v>45874.28875651701</v>
       </c>
       <c r="C17" t="n">
-        <v>0.02421041698445367</v>
+        <v>0.02526132685750728</v>
       </c>
       <c r="D17" t="n">
-        <v>6051.607763465174</v>
+        <v>5704.904184210594</v>
       </c>
       <c r="E17" t="n">
-        <v>86515.13008946966</v>
+        <v>86043.67332882342</v>
       </c>
     </row>
     <row r="18">
@@ -1713,16 +1713,16 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>-1216.285465580579</v>
+        <v>-1206.439233822232</v>
       </c>
       <c r="C18" t="n">
-        <v>0.05708036665229766</v>
+        <v>0.05883483463971662</v>
       </c>
       <c r="D18" t="n">
-        <v>-2469.279667582122</v>
+        <v>-2458.041059675247</v>
       </c>
       <c r="E18" t="n">
-        <v>36.70873642096376</v>
+        <v>45.16259203078357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>